<commit_message>
chore(terms): update custom translation terminology
</commit_message>
<xml_diff>
--- a/custom_terms.xlsx
+++ b/custom_terms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Apps\VideoLingo-inspect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3FA740-08C9-4E73-8958-DD3433E959F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D75DCA7-F36A-430E-89EA-6052E3E35B36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10080" yWindow="2430" windowWidth="26200" windowHeight="18470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1280" yWindow="460" windowWidth="28460" windowHeight="19740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="terminology" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>Source</t>
   </si>
@@ -111,13 +111,28 @@
   </si>
   <si>
     <t>机匣</t>
+  </si>
+  <si>
+    <t>forgottenWeapons.com</t>
+  </si>
+  <si>
+    <t>被遗忘的武器</t>
+  </si>
+  <si>
+    <t>Forgotten Weapons</t>
+  </si>
+  <si>
+    <t>Ian McCollum</t>
+  </si>
+  <si>
+    <t>伊恩麦柯莱姆</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,6 +146,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -155,11 +175,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -650,7 +673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="9.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="28.26953125" customWidth="1"/>
@@ -766,6 +789,30 @@
         <v>25</v>
       </c>
     </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>